<commit_message>
Reemplaza Cintia Vidal por Catalina Linette
</commit_message>
<xml_diff>
--- a/horarios.xlsx
+++ b/horarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dreame\Desktop\Claude\Dreame\Turnos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4627F12C-69C9-4F18-9B18-FDB818431D36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1D7DA2-0C7B-4EB7-A371-D49520DEB05C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -89,9 +89,6 @@
     <t>LISSETTE MORALES</t>
   </si>
   <si>
-    <t>CINTIA VIDAL</t>
-  </si>
-  <si>
     <t>JORDAN RIMMELIN</t>
   </si>
   <si>
@@ -105,6 +102,9 @@
   </si>
   <si>
     <t>Semana 44</t>
+  </si>
+  <si>
+    <t>CATALINA LINETTE</t>
   </si>
 </sst>
 </file>
@@ -1127,7 +1127,7 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>13</v>
@@ -1174,7 +1174,7 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B17" s="2">
         <v>0.45833333333333331</v>
@@ -1221,7 +1221,7 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B19" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -1880,7 +1880,7 @@
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B34" s="2">
         <v>0.41666666666666669</v>
@@ -1927,7 +1927,7 @@
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B35" s="2">
         <v>0.41666666666666669</v>
@@ -1974,7 +1974,7 @@
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B37" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
@@ -2633,7 +2633,7 @@
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>5</v>
@@ -2680,7 +2680,7 @@
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>5</v>
@@ -2727,7 +2727,7 @@
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B55" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C55" s="4"/>
       <c r="D55" s="4"/>
@@ -3386,7 +3386,7 @@
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B70" s="2">
         <v>0.45833333333333331</v>
@@ -3433,7 +3433,7 @@
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B71" s="2">
         <v>0.45833333333333331</v>
@@ -3480,7 +3480,7 @@
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B73" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
@@ -4139,7 +4139,7 @@
     </row>
     <row r="88" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B88" s="2">
         <v>0.45833333333333331</v>
@@ -4186,7 +4186,7 @@
     </row>
     <row r="89" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B89" s="2">
         <v>0.45833333333333331</v>

</xml_diff>

<commit_message>
Actualiza horarios 16-oct: Camila Soto cubre vacantes, ajuste Catalina Linette
</commit_message>
<xml_diff>
--- a/horarios.xlsx
+++ b/horarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dreame\Desktop\Claude\Dreame\Turnos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1D7DA2-0C7B-4EB7-A371-D49520DEB05C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0E1E667-F2A9-4E68-8034-01B845B14671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Octubre" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -71,9 +72,6 @@
     <t>DIEGO MARTINEZ</t>
   </si>
   <si>
-    <t>VACANTE</t>
-  </si>
-  <si>
     <t>ID Inactivo</t>
   </si>
   <si>
@@ -105,6 +103,9 @@
   </si>
   <si>
     <t>CATALINA LINETTE</t>
+  </si>
+  <si>
+    <t>CAMILA SOTO</t>
   </si>
 </sst>
 </file>
@@ -151,11 +152,11 @@
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="16" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -467,7 +468,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="4"/>
@@ -488,31 +489,31 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="5">
         <v>46293</v>
       </c>
       <c r="C2" s="4"/>
-      <c r="D2" s="3">
+      <c r="D2" s="5">
         <v>46294</v>
       </c>
       <c r="E2" s="4"/>
-      <c r="F2" s="3">
+      <c r="F2" s="5">
         <v>46295</v>
       </c>
       <c r="G2" s="4"/>
-      <c r="H2" s="3">
+      <c r="H2" s="5">
         <v>46296</v>
       </c>
       <c r="I2" s="4"/>
-      <c r="J2" s="3">
+      <c r="J2" s="5">
         <v>46297</v>
       </c>
       <c r="K2" s="4"/>
-      <c r="L2" s="3">
+      <c r="L2" s="5">
         <v>46298</v>
       </c>
       <c r="M2" s="4"/>
-      <c r="N2" s="3">
+      <c r="N2" s="5">
         <v>46299</v>
       </c>
       <c r="O2" s="4"/>
@@ -892,13 +893,13 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="C11" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>5</v>
@@ -913,10 +914,10 @@
         <v>5</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J11" s="2">
         <v>0.4375</v>
@@ -939,7 +940,7 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" s="2">
         <v>0.45833333333333331</v>
@@ -986,7 +987,7 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13" s="2">
         <v>0.45833333333333331</v>
@@ -1033,7 +1034,7 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14" s="2">
         <v>0.45833333333333331</v>
@@ -1080,7 +1081,7 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" s="2">
         <v>0.45833333333333331</v>
@@ -1127,13 +1128,13 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>5</v>
@@ -1148,10 +1149,10 @@
         <v>5</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J16" s="2">
         <v>0.4375</v>
@@ -1174,54 +1175,54 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="2">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="C17" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H17" s="2">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="I17" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="J17" s="2">
+        <v>0.4375</v>
+      </c>
+      <c r="K17" s="2">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="L17" s="2">
+        <v>0.4375</v>
+      </c>
+      <c r="M17" s="2">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="N17" s="2">
+        <v>0.4375</v>
+      </c>
+      <c r="O17" s="2">
+        <v>0.85416666666666663</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="B19" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="B17" s="2">
-        <v>0.45833333333333331</v>
-      </c>
-      <c r="C17" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="H17" s="2">
-        <v>0.45833333333333331</v>
-      </c>
-      <c r="I17" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="J17" s="2">
-        <v>0.4375</v>
-      </c>
-      <c r="K17" s="2">
-        <v>0.85416666666666663</v>
-      </c>
-      <c r="L17" s="2">
-        <v>0.4375</v>
-      </c>
-      <c r="M17" s="2">
-        <v>0.85416666666666663</v>
-      </c>
-      <c r="N17" s="2">
-        <v>0.4375</v>
-      </c>
-      <c r="O17" s="2">
-        <v>0.85416666666666663</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B19" s="5" t="s">
-        <v>19</v>
       </c>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
@@ -1241,31 +1242,31 @@
       <c r="A20" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B20" s="3">
+      <c r="B20" s="5">
         <v>46300</v>
       </c>
       <c r="C20" s="4"/>
-      <c r="D20" s="3">
+      <c r="D20" s="5">
         <v>46301</v>
       </c>
       <c r="E20" s="4"/>
-      <c r="F20" s="3">
+      <c r="F20" s="5">
         <v>46302</v>
       </c>
       <c r="G20" s="4"/>
-      <c r="H20" s="3">
+      <c r="H20" s="5">
         <v>46303</v>
       </c>
       <c r="I20" s="4"/>
-      <c r="J20" s="3">
+      <c r="J20" s="5">
         <v>46304</v>
       </c>
       <c r="K20" s="4"/>
-      <c r="L20" s="3">
+      <c r="L20" s="5">
         <v>46305</v>
       </c>
       <c r="M20" s="4"/>
-      <c r="N20" s="3">
+      <c r="N20" s="5">
         <v>46306</v>
       </c>
       <c r="O20" s="4"/>
@@ -1645,7 +1646,7 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="B29" s="2">
         <v>0.41666666666666669</v>
@@ -1692,7 +1693,7 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B30" s="2">
         <v>0.41666666666666669</v>
@@ -1739,7 +1740,7 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B31" s="2">
         <v>0.41666666666666669</v>
@@ -1786,7 +1787,7 @@
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B32" s="2">
         <v>0.4375</v>
@@ -1833,7 +1834,7 @@
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B33" s="2">
         <v>0.41666666666666669</v>
@@ -1880,7 +1881,7 @@
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B34" s="2">
         <v>0.41666666666666669</v>
@@ -1927,7 +1928,7 @@
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B35" s="2">
         <v>0.41666666666666669</v>
@@ -1973,8 +1974,8 @@
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B37" s="5" t="s">
-        <v>20</v>
+      <c r="B37" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
@@ -1994,31 +1995,31 @@
       <c r="A38" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B38" s="3">
+      <c r="B38" s="5">
         <v>46307</v>
       </c>
       <c r="C38" s="4"/>
-      <c r="D38" s="3">
+      <c r="D38" s="5">
         <v>46308</v>
       </c>
       <c r="E38" s="4"/>
-      <c r="F38" s="3">
+      <c r="F38" s="5">
         <v>46309</v>
       </c>
       <c r="G38" s="4"/>
-      <c r="H38" s="3">
+      <c r="H38" s="5">
         <v>46310</v>
       </c>
       <c r="I38" s="4"/>
-      <c r="J38" s="3">
+      <c r="J38" s="5">
         <v>46311</v>
       </c>
       <c r="K38" s="4"/>
-      <c r="L38" s="3">
+      <c r="L38" s="5">
         <v>46312</v>
       </c>
       <c r="M38" s="4"/>
-      <c r="N38" s="3">
+      <c r="N38" s="5">
         <v>46313</v>
       </c>
       <c r="O38" s="4"/>
@@ -2398,7 +2399,7 @@
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>5</v>
@@ -2445,7 +2446,7 @@
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>5</v>
@@ -2492,7 +2493,7 @@
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>5</v>
@@ -2539,7 +2540,7 @@
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>5</v>
@@ -2586,7 +2587,7 @@
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>5</v>
@@ -2633,7 +2634,7 @@
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>5</v>
@@ -2680,7 +2681,7 @@
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>5</v>
@@ -2726,8 +2727,8 @@
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B55" s="5" t="s">
-        <v>21</v>
+      <c r="B55" s="3" t="s">
+        <v>20</v>
       </c>
       <c r="C55" s="4"/>
       <c r="D55" s="4"/>
@@ -2747,31 +2748,31 @@
       <c r="A56" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B56" s="3">
+      <c r="B56" s="5">
         <v>46314</v>
       </c>
       <c r="C56" s="4"/>
-      <c r="D56" s="3">
+      <c r="D56" s="5">
         <v>46315</v>
       </c>
       <c r="E56" s="4"/>
-      <c r="F56" s="3">
+      <c r="F56" s="5">
         <v>46316</v>
       </c>
       <c r="G56" s="4"/>
-      <c r="H56" s="3">
+      <c r="H56" s="5">
         <v>46317</v>
       </c>
       <c r="I56" s="4"/>
-      <c r="J56" s="3">
+      <c r="J56" s="5">
         <v>46318</v>
       </c>
       <c r="K56" s="4"/>
-      <c r="L56" s="3">
+      <c r="L56" s="5">
         <v>46319</v>
       </c>
       <c r="M56" s="4"/>
-      <c r="N56" s="3">
+      <c r="N56" s="5">
         <v>46320</v>
       </c>
       <c r="O56" s="4"/>
@@ -3151,7 +3152,7 @@
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="B65" s="2">
         <v>0.45833333333333331</v>
@@ -3198,7 +3199,7 @@
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B66" s="2">
         <v>0.45833333333333331</v>
@@ -3245,7 +3246,7 @@
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B67" s="2">
         <v>0.45833333333333331</v>
@@ -3292,7 +3293,7 @@
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B68" s="2">
         <v>0.45833333333333331</v>
@@ -3339,7 +3340,7 @@
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B69" s="2">
         <v>0.45833333333333331</v>
@@ -3386,7 +3387,7 @@
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B70" s="2">
         <v>0.45833333333333331</v>
@@ -3394,11 +3395,11 @@
       <c r="C70" s="2">
         <v>0.79166666666666663</v>
       </c>
-      <c r="D70" s="2">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="E70" s="2">
-        <v>0.79166666666666663</v>
+      <c r="D70" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E70" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="F70" s="2" t="s">
         <v>5</v>
@@ -3406,11 +3407,11 @@
       <c r="G70" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H70" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I70" s="2" t="s">
-        <v>5</v>
+      <c r="H70" s="2">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I70" s="2">
+        <v>0.79166666666666663</v>
       </c>
       <c r="J70" s="2">
         <v>0.41666666666666669</v>
@@ -3433,7 +3434,7 @@
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B71" s="2">
         <v>0.45833333333333331</v>
@@ -3479,8 +3480,8 @@
       </c>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B73" s="5" t="s">
-        <v>22</v>
+      <c r="B73" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="C73" s="4"/>
       <c r="D73" s="4"/>
@@ -3500,31 +3501,31 @@
       <c r="A74" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B74" s="3">
+      <c r="B74" s="5">
         <v>46321</v>
       </c>
       <c r="C74" s="4"/>
-      <c r="D74" s="3">
+      <c r="D74" s="5">
         <v>46322</v>
       </c>
       <c r="E74" s="4"/>
-      <c r="F74" s="3">
+      <c r="F74" s="5">
         <v>46323</v>
       </c>
       <c r="G74" s="4"/>
-      <c r="H74" s="3">
+      <c r="H74" s="5">
         <v>46324</v>
       </c>
       <c r="I74" s="4"/>
-      <c r="J74" s="3">
+      <c r="J74" s="5">
         <v>46325</v>
       </c>
       <c r="K74" s="4"/>
-      <c r="L74" s="3">
+      <c r="L74" s="5">
         <v>46326</v>
       </c>
       <c r="M74" s="4"/>
-      <c r="N74" s="3">
+      <c r="N74" s="5">
         <v>46327</v>
       </c>
       <c r="O74" s="4"/>
@@ -3904,7 +3905,7 @@
     </row>
     <row r="83" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="B83" s="2">
         <v>0.45833333333333331</v>
@@ -3951,7 +3952,7 @@
     </row>
     <row r="84" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B84" s="2">
         <v>0.45833333333333331</v>
@@ -3998,7 +3999,7 @@
     </row>
     <row r="85" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B85" s="2">
         <v>0.45833333333333331</v>
@@ -4045,7 +4046,7 @@
     </row>
     <row r="86" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B86" s="2">
         <v>0.45833333333333331</v>
@@ -4092,7 +4093,7 @@
     </row>
     <row r="87" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B87" s="2">
         <v>0.45833333333333331</v>
@@ -4139,7 +4140,7 @@
     </row>
     <row r="88" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B88" s="2">
         <v>0.45833333333333331</v>
@@ -4186,7 +4187,7 @@
     </row>
     <row r="89" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B89" s="2">
         <v>0.45833333333333331</v>
@@ -4233,6 +4234,30 @@
     </row>
   </sheetData>
   <mergeCells count="40">
+    <mergeCell ref="H56:I56"/>
+    <mergeCell ref="N56:O56"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="N20:O20"/>
+    <mergeCell ref="J38:K38"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="J74:K74"/>
+    <mergeCell ref="L74:M74"/>
+    <mergeCell ref="B73:O73"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="F56:G56"/>
+    <mergeCell ref="J56:K56"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="L56:M56"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="B55:O55"/>
+    <mergeCell ref="N74:O74"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="F74:G74"/>
+    <mergeCell ref="H74:I74"/>
     <mergeCell ref="B1:O1"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="F2:G2"/>
@@ -4249,30 +4274,6 @@
     <mergeCell ref="D38:E38"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="J74:K74"/>
-    <mergeCell ref="L74:M74"/>
-    <mergeCell ref="B73:O73"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="F56:G56"/>
-    <mergeCell ref="J56:K56"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="L56:M56"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="B55:O55"/>
-    <mergeCell ref="N74:O74"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="F74:G74"/>
-    <mergeCell ref="H74:I74"/>
-    <mergeCell ref="H56:I56"/>
-    <mergeCell ref="N56:O56"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="H38:I38"/>
-    <mergeCell ref="N20:O20"/>
-    <mergeCell ref="J38:K38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualiza horarios 16-oct: ajuste turno Geisslen Erices
</commit_message>
<xml_diff>
--- a/horarios.xlsx
+++ b/horarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dreame\Desktop\Claude\Dreame\Turnos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0E1E667-F2A9-4E68-8034-01B845B14671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B3288F0-6BE6-4712-955E-17A90122428A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3772,11 +3772,11 @@
       <c r="C80" s="2">
         <v>0.83333333333333337</v>
       </c>
-      <c r="D80" s="2">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="E80" s="2">
-        <v>0.83333333333333337</v>
+      <c r="D80" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="F80" s="2" t="s">
         <v>5</v>
@@ -3784,11 +3784,11 @@
       <c r="G80" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H80" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I80" s="2" t="s">
-        <v>5</v>
+      <c r="H80" s="2">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I80" s="2">
+        <v>0.83333333333333337</v>
       </c>
       <c r="J80" s="2">
         <v>0.41666666666666669</v>

</xml_diff>

<commit_message>
Actualiza horarios 16-oct: ajuste turno Camila Soto
</commit_message>
<xml_diff>
--- a/horarios.xlsx
+++ b/horarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dreame\Desktop\Claude\Dreame\Turnos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B3288F0-6BE6-4712-955E-17A90122428A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89360B60-1D5C-43FD-B17F-13F86FB5A00E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -126,12 +126,18 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -146,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -157,6 +163,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="20" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3903,50 +3913,50 @@
         <v>0.83333333333333337</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
+    <row r="83" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B83" s="2">
-        <v>0.45833333333333331</v>
-      </c>
-      <c r="C83" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D83" s="2">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="E83" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="F83" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G83" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="H83" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I83" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="J83" s="2">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K83" s="2">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L83" s="2">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M83" s="2">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N83" s="2">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="O83" s="2">
+      <c r="B83" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C83" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D83" s="7">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E83" s="7">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F83" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G83" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="H83" s="7">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="I83" s="7">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="J83" s="7">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K83" s="7">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L83" s="7">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M83" s="7">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N83" s="7">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="O83" s="7">
         <v>0.83333333333333337</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualiza horarios 24-oct: ajuste turno Catalina Linette (semana 44)
</commit_message>
<xml_diff>
--- a/horarios.xlsx
+++ b/horarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dreame\Desktop\Claude\Dreame\Turnos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89360B60-1D5C-43FD-B17F-13F86FB5A00E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CDDFBA6-1829-47D5-B368-083DBF8589BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Octubre" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -158,15 +157,15 @@
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="20" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="16" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="20" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -478,22 +477,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -502,31 +501,31 @@
       <c r="B2" s="5">
         <v>46293</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="6"/>
       <c r="D2" s="5">
         <v>46294</v>
       </c>
-      <c r="E2" s="4"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="5">
         <v>46295</v>
       </c>
-      <c r="G2" s="4"/>
+      <c r="G2" s="6"/>
       <c r="H2" s="5">
         <v>46296</v>
       </c>
-      <c r="I2" s="4"/>
+      <c r="I2" s="6"/>
       <c r="J2" s="5">
         <v>46297</v>
       </c>
-      <c r="K2" s="4"/>
+      <c r="K2" s="6"/>
       <c r="L2" s="5">
         <v>46298</v>
       </c>
-      <c r="M2" s="4"/>
+      <c r="M2" s="6"/>
       <c r="N2" s="5">
         <v>46299</v>
       </c>
-      <c r="O2" s="4"/>
+      <c r="O2" s="6"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1231,22 +1230,22 @@
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
-      <c r="M19" s="4"/>
-      <c r="N19" s="4"/>
-      <c r="O19" s="4"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="6"/>
+      <c r="M19" s="6"/>
+      <c r="N19" s="6"/>
+      <c r="O19" s="6"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
@@ -1255,31 +1254,31 @@
       <c r="B20" s="5">
         <v>46300</v>
       </c>
-      <c r="C20" s="4"/>
+      <c r="C20" s="6"/>
       <c r="D20" s="5">
         <v>46301</v>
       </c>
-      <c r="E20" s="4"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="5">
         <v>46302</v>
       </c>
-      <c r="G20" s="4"/>
+      <c r="G20" s="6"/>
       <c r="H20" s="5">
         <v>46303</v>
       </c>
-      <c r="I20" s="4"/>
+      <c r="I20" s="6"/>
       <c r="J20" s="5">
         <v>46304</v>
       </c>
-      <c r="K20" s="4"/>
+      <c r="K20" s="6"/>
       <c r="L20" s="5">
         <v>46305</v>
       </c>
-      <c r="M20" s="4"/>
+      <c r="M20" s="6"/>
       <c r="N20" s="5">
         <v>46306</v>
       </c>
-      <c r="O20" s="4"/>
+      <c r="O20" s="6"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
@@ -1984,22 +1983,22 @@
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4"/>
-      <c r="I37" s="4"/>
-      <c r="J37" s="4"/>
-      <c r="K37" s="4"/>
-      <c r="L37" s="4"/>
-      <c r="M37" s="4"/>
-      <c r="N37" s="4"/>
-      <c r="O37" s="4"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="6"/>
+      <c r="J37" s="6"/>
+      <c r="K37" s="6"/>
+      <c r="L37" s="6"/>
+      <c r="M37" s="6"/>
+      <c r="N37" s="6"/>
+      <c r="O37" s="6"/>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
@@ -2008,31 +2007,31 @@
       <c r="B38" s="5">
         <v>46307</v>
       </c>
-      <c r="C38" s="4"/>
+      <c r="C38" s="6"/>
       <c r="D38" s="5">
         <v>46308</v>
       </c>
-      <c r="E38" s="4"/>
+      <c r="E38" s="6"/>
       <c r="F38" s="5">
         <v>46309</v>
       </c>
-      <c r="G38" s="4"/>
+      <c r="G38" s="6"/>
       <c r="H38" s="5">
         <v>46310</v>
       </c>
-      <c r="I38" s="4"/>
+      <c r="I38" s="6"/>
       <c r="J38" s="5">
         <v>46311</v>
       </c>
-      <c r="K38" s="4"/>
+      <c r="K38" s="6"/>
       <c r="L38" s="5">
         <v>46312</v>
       </c>
-      <c r="M38" s="4"/>
+      <c r="M38" s="6"/>
       <c r="N38" s="5">
         <v>46313</v>
       </c>
-      <c r="O38" s="4"/>
+      <c r="O38" s="6"/>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B39" s="1" t="s">
@@ -2737,22 +2736,22 @@
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B55" s="3" t="s">
+      <c r="B55" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C55" s="4"/>
-      <c r="D55" s="4"/>
-      <c r="E55" s="4"/>
-      <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
-      <c r="H55" s="4"/>
-      <c r="I55" s="4"/>
-      <c r="J55" s="4"/>
-      <c r="K55" s="4"/>
-      <c r="L55" s="4"/>
-      <c r="M55" s="4"/>
-      <c r="N55" s="4"/>
-      <c r="O55" s="4"/>
+      <c r="C55" s="6"/>
+      <c r="D55" s="6"/>
+      <c r="E55" s="6"/>
+      <c r="F55" s="6"/>
+      <c r="G55" s="6"/>
+      <c r="H55" s="6"/>
+      <c r="I55" s="6"/>
+      <c r="J55" s="6"/>
+      <c r="K55" s="6"/>
+      <c r="L55" s="6"/>
+      <c r="M55" s="6"/>
+      <c r="N55" s="6"/>
+      <c r="O55" s="6"/>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
@@ -2761,31 +2760,31 @@
       <c r="B56" s="5">
         <v>46314</v>
       </c>
-      <c r="C56" s="4"/>
+      <c r="C56" s="6"/>
       <c r="D56" s="5">
         <v>46315</v>
       </c>
-      <c r="E56" s="4"/>
+      <c r="E56" s="6"/>
       <c r="F56" s="5">
         <v>46316</v>
       </c>
-      <c r="G56" s="4"/>
+      <c r="G56" s="6"/>
       <c r="H56" s="5">
         <v>46317</v>
       </c>
-      <c r="I56" s="4"/>
+      <c r="I56" s="6"/>
       <c r="J56" s="5">
         <v>46318</v>
       </c>
-      <c r="K56" s="4"/>
+      <c r="K56" s="6"/>
       <c r="L56" s="5">
         <v>46319</v>
       </c>
-      <c r="M56" s="4"/>
+      <c r="M56" s="6"/>
       <c r="N56" s="5">
         <v>46320</v>
       </c>
-      <c r="O56" s="4"/>
+      <c r="O56" s="6"/>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B57" s="1" t="s">
@@ -3490,22 +3489,22 @@
       </c>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B73" s="3" t="s">
+      <c r="B73" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C73" s="4"/>
-      <c r="D73" s="4"/>
-      <c r="E73" s="4"/>
-      <c r="F73" s="4"/>
-      <c r="G73" s="4"/>
-      <c r="H73" s="4"/>
-      <c r="I73" s="4"/>
-      <c r="J73" s="4"/>
-      <c r="K73" s="4"/>
-      <c r="L73" s="4"/>
-      <c r="M73" s="4"/>
-      <c r="N73" s="4"/>
-      <c r="O73" s="4"/>
+      <c r="C73" s="6"/>
+      <c r="D73" s="6"/>
+      <c r="E73" s="6"/>
+      <c r="F73" s="6"/>
+      <c r="G73" s="6"/>
+      <c r="H73" s="6"/>
+      <c r="I73" s="6"/>
+      <c r="J73" s="6"/>
+      <c r="K73" s="6"/>
+      <c r="L73" s="6"/>
+      <c r="M73" s="6"/>
+      <c r="N73" s="6"/>
+      <c r="O73" s="6"/>
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
@@ -3514,31 +3513,31 @@
       <c r="B74" s="5">
         <v>46321</v>
       </c>
-      <c r="C74" s="4"/>
+      <c r="C74" s="6"/>
       <c r="D74" s="5">
         <v>46322</v>
       </c>
-      <c r="E74" s="4"/>
+      <c r="E74" s="6"/>
       <c r="F74" s="5">
         <v>46323</v>
       </c>
-      <c r="G74" s="4"/>
+      <c r="G74" s="6"/>
       <c r="H74" s="5">
         <v>46324</v>
       </c>
-      <c r="I74" s="4"/>
+      <c r="I74" s="6"/>
       <c r="J74" s="5">
         <v>46325</v>
       </c>
-      <c r="K74" s="4"/>
+      <c r="K74" s="6"/>
       <c r="L74" s="5">
         <v>46326</v>
       </c>
-      <c r="M74" s="4"/>
+      <c r="M74" s="6"/>
       <c r="N74" s="5">
         <v>46327</v>
       </c>
-      <c r="O74" s="4"/>
+      <c r="O74" s="6"/>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B75" s="1" t="s">
@@ -3913,50 +3912,50 @@
         <v>0.83333333333333337</v>
       </c>
     </row>
-    <row r="83" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="6" t="s">
+    <row r="83" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B83" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C83" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D83" s="7">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="E83" s="7">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="F83" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="G83" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="H83" s="7">
-        <v>0.45833333333333331</v>
-      </c>
-      <c r="I83" s="7">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="J83" s="7">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K83" s="7">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L83" s="7">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M83" s="7">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N83" s="7">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="O83" s="7">
+      <c r="B83" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D83" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E83" s="4">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F83" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G83" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H83" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="I83" s="4">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="J83" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K83" s="4">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L83" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M83" s="4">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N83" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="O83" s="4">
         <v>0.83333333333333337</v>
       </c>
     </row>
@@ -4159,10 +4158,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D88" s="2">
-        <v>0.41666666666666669</v>
+        <v>0.4375</v>
       </c>
       <c r="E88" s="2">
-        <v>0.79166666666666663</v>
+        <v>0.85416666666666663</v>
       </c>
       <c r="F88" s="2" t="s">
         <v>5</v>
@@ -4177,19 +4176,19 @@
         <v>5</v>
       </c>
       <c r="J88" s="2">
-        <v>0.41666666666666669</v>
+        <v>0.4375</v>
       </c>
       <c r="K88" s="2">
-        <v>0.83333333333333337</v>
+        <v>0.85416666666666663</v>
       </c>
       <c r="L88" s="2">
-        <v>0.41666666666666669</v>
+        <v>0.4375</v>
       </c>
       <c r="M88" s="2">
-        <v>0.83333333333333337</v>
+        <v>0.85416666666666663</v>
       </c>
       <c r="N88" s="2">
-        <v>0.41666666666666669</v>
+        <v>0.45833333333333331</v>
       </c>
       <c r="O88" s="2">
         <v>0.83333333333333337</v>
@@ -4244,30 +4243,6 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="H56:I56"/>
-    <mergeCell ref="N56:O56"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="H38:I38"/>
-    <mergeCell ref="N20:O20"/>
-    <mergeCell ref="J38:K38"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="J74:K74"/>
-    <mergeCell ref="L74:M74"/>
-    <mergeCell ref="B73:O73"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="F56:G56"/>
-    <mergeCell ref="J56:K56"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="L56:M56"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="B55:O55"/>
-    <mergeCell ref="N74:O74"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="F74:G74"/>
-    <mergeCell ref="H74:I74"/>
     <mergeCell ref="B1:O1"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="F2:G2"/>
@@ -4284,6 +4259,30 @@
     <mergeCell ref="D38:E38"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
+    <mergeCell ref="J74:K74"/>
+    <mergeCell ref="L74:M74"/>
+    <mergeCell ref="B73:O73"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="F56:G56"/>
+    <mergeCell ref="J56:K56"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="L56:M56"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="N74:O74"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="F74:G74"/>
+    <mergeCell ref="H74:I74"/>
+    <mergeCell ref="H56:I56"/>
+    <mergeCell ref="N56:O56"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="N20:O20"/>
+    <mergeCell ref="J38:K38"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="B55:O55"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>